<commit_message>
Single Flow Run and Report Feature added
</commit_message>
<xml_diff>
--- a/TestData/ExampleData.xlsx
+++ b/TestData/ExampleData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MaestroLab\Maestro-Excel-Data-Driven-Framework\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\AppData\Local\Programs\Maestro Studio\Maestro\Test\Maestro-Excel-Data-Driven-Framework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBA394D-8258-4C98-851F-E7264EAB3953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96728D42-D4AF-4724-9159-21E9EDC292EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="878" activeTab="1" xr2:uid="{8F7D7BB0-42BA-4985-9199-EDA16EBB489C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="878" xr2:uid="{8F7D7BB0-42BA-4985-9199-EDA16EBB489C}"/>
   </bookViews>
   <sheets>
     <sheet name="Example_LoginData" sheetId="12" r:id="rId1"/>

</xml_diff>